<commit_message>
Link operator and mTLS features to governing specs
</commit_message>
<xml_diff>
--- a/.ssot/reports/feature-governance-link-matrix.xlsx
+++ b/.ssot/reports/feature-governance-link-matrix.xlsx
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -2507,7 +2507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC78"/>
+  <dimension ref="A1:BF78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2565,6 +2565,9 @@
     <col width="10" customWidth="1" min="53" max="53"/>
     <col width="10" customWidth="1" min="54" max="54"/>
     <col width="10" customWidth="1" min="55" max="55"/>
+    <col width="10" customWidth="1" min="56" max="56"/>
+    <col width="10" customWidth="1" min="57" max="57"/>
+    <col width="10" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2750,95 +2753,110 @@
       </c>
       <c r="AK1" t="inlineStr">
         <is>
+          <t>spc:2078</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>spc:2080</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
           <t>spc:2084</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>spc:2085</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>spc:2086</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>spc:2088</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>spc:2093</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>spc:2097</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>spc:2098</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>spc:2099</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>spc:2100</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>spc:2101</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>spc:2102</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>spc:2103</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>spc:2104</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>spc:2109</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>spc:2114</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>spc:2115</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>spc:2117</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>spc:2119</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>spc:2123</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
         <is>
           <t>spc:2142</t>
         </is>
@@ -2920,6 +2938,9 @@
       <c r="BA2" t="inlineStr"/>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2987,20 +3008,23 @@
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AT3" t="inlineStr"/>
       <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AW3" t="inlineStr"/>
       <c r="AX3" t="inlineStr"/>
       <c r="AY3" t="inlineStr"/>
       <c r="AZ3" t="inlineStr"/>
       <c r="BA3" t="inlineStr"/>
       <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr">
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3067,13 +3091,13 @@
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr"/>
       <c r="AT4" t="inlineStr"/>
@@ -3086,6 +3110,9 @@
       <c r="BA4" t="inlineStr"/>
       <c r="BB4" t="inlineStr"/>
       <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3148,13 +3175,13 @@
       <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr"/>
-      <c r="AQ5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr"/>
       <c r="AT5" t="inlineStr"/>
@@ -3167,6 +3194,9 @@
       <c r="BA5" t="inlineStr"/>
       <c r="BB5" t="inlineStr"/>
       <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3229,13 +3259,13 @@
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr"/>
@@ -3248,6 +3278,9 @@
       <c r="BA6" t="inlineStr"/>
       <c r="BB6" t="inlineStr"/>
       <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3310,13 +3343,13 @@
       <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
@@ -3329,6 +3362,9 @@
       <c r="BA7" t="inlineStr"/>
       <c r="BB7" t="inlineStr"/>
       <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3391,13 +3427,13 @@
       <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="inlineStr"/>
@@ -3410,6 +3446,9 @@
       <c r="BA8" t="inlineStr"/>
       <c r="BB8" t="inlineStr"/>
       <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3472,13 +3511,13 @@
       <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="inlineStr"/>
@@ -3491,6 +3530,9 @@
       <c r="BA9" t="inlineStr"/>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3553,13 +3595,13 @@
       <c r="AL10" t="inlineStr"/>
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="inlineStr"/>
@@ -3572,6 +3614,9 @@
       <c r="BA10" t="inlineStr"/>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3590,7 +3635,11 @@
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
@@ -3649,6 +3698,9 @@
       <c r="BA11" t="inlineStr"/>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3718,14 +3770,17 @@
       <c r="AW12" t="inlineStr"/>
       <c r="AX12" t="inlineStr"/>
       <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AZ12" t="inlineStr"/>
       <c r="BA12" t="inlineStr"/>
-      <c r="BB12" t="inlineStr"/>
-      <c r="BC12" t="inlineStr">
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3787,18 +3842,18 @@
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AS13" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AV13" t="inlineStr"/>
       <c r="AW13" t="inlineStr"/>
       <c r="AX13" t="inlineStr"/>
@@ -3806,7 +3861,10 @@
       <c r="AZ13" t="inlineStr"/>
       <c r="BA13" t="inlineStr"/>
       <c r="BB13" t="inlineStr"/>
-      <c r="BC13" t="inlineStr">
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -3829,7 +3887,11 @@
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -3844,7 +3906,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
@@ -3872,34 +3938,37 @@
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr"/>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="AU14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AV14" t="inlineStr"/>
-      <c r="AW14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AX14" t="inlineStr"/>
       <c r="AY14" t="inlineStr"/>
-      <c r="AZ14" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AZ14" t="inlineStr"/>
       <c r="BA14" t="inlineStr"/>
-      <c r="BB14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3964,19 +4033,22 @@
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="inlineStr"/>
-      <c r="AU15" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AU15" t="inlineStr"/>
       <c r="AV15" t="inlineStr"/>
-      <c r="AW15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AX15" t="inlineStr"/>
       <c r="AY15" t="inlineStr"/>
       <c r="AZ15" t="inlineStr"/>
       <c r="BA15" t="inlineStr"/>
       <c r="BB15" t="inlineStr"/>
-      <c r="BC15" t="inlineStr">
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4037,18 +4109,18 @@
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr"/>
       <c r="AP16" t="inlineStr"/>
-      <c r="AQ16" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AS16" t="inlineStr"/>
-      <c r="AT16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AU16" t="inlineStr"/>
       <c r="AV16" t="inlineStr"/>
       <c r="AW16" t="inlineStr"/>
@@ -4057,7 +4129,10 @@
       <c r="AZ16" t="inlineStr"/>
       <c r="BA16" t="inlineStr"/>
       <c r="BB16" t="inlineStr"/>
-      <c r="BC16" t="inlineStr">
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4125,20 +4200,23 @@
       <c r="AQ17" t="inlineStr"/>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="inlineStr"/>
-      <c r="AT17" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AT17" t="inlineStr"/>
       <c r="AU17" t="inlineStr"/>
-      <c r="AV17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AW17" t="inlineStr"/>
       <c r="AX17" t="inlineStr"/>
       <c r="AY17" t="inlineStr"/>
       <c r="AZ17" t="inlineStr"/>
       <c r="BA17" t="inlineStr"/>
       <c r="BB17" t="inlineStr"/>
-      <c r="BC17" t="inlineStr">
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4199,11 +4277,7 @@
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr"/>
       <c r="AP18" t="inlineStr"/>
-      <c r="AQ18" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AQ18" t="inlineStr"/>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="inlineStr">
         <is>
@@ -4211,19 +4285,26 @@
         </is>
       </c>
       <c r="AT18" t="inlineStr"/>
-      <c r="AU18" t="inlineStr"/>
-      <c r="AV18" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr"/>
       <c r="AW18" t="inlineStr"/>
-      <c r="AX18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AY18" t="inlineStr"/>
       <c r="AZ18" t="inlineStr"/>
       <c r="BA18" t="inlineStr"/>
       <c r="BB18" t="inlineStr"/>
-      <c r="BC18" t="inlineStr">
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4294,17 +4375,20 @@
       <c r="AX19" t="inlineStr"/>
       <c r="AY19" t="inlineStr"/>
       <c r="AZ19" t="inlineStr"/>
-      <c r="BA19" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="BB19" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
       <c r="BC19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="BD19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4390,6 +4474,9 @@
       <c r="BA20" t="inlineStr"/>
       <c r="BB20" t="inlineStr"/>
       <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+      <c r="BE20" t="inlineStr"/>
+      <c r="BF20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4408,7 +4495,11 @@
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
@@ -4471,6 +4562,9 @@
       <c r="BA21" t="inlineStr"/>
       <c r="BB21" t="inlineStr"/>
       <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4546,20 +4640,23 @@
       <c r="AQ22" t="inlineStr"/>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="inlineStr"/>
-      <c r="AT22" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AT22" t="inlineStr"/>
       <c r="AU22" t="inlineStr"/>
-      <c r="AV22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AW22" t="inlineStr"/>
       <c r="AX22" t="inlineStr"/>
       <c r="AY22" t="inlineStr"/>
       <c r="AZ22" t="inlineStr"/>
       <c r="BA22" t="inlineStr"/>
       <c r="BB22" t="inlineStr"/>
-      <c r="BC22" t="inlineStr">
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr"/>
+      <c r="BE22" t="inlineStr"/>
+      <c r="BF22" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4641,6 +4738,9 @@
       <c r="BA23" t="inlineStr"/>
       <c r="BB23" t="inlineStr"/>
       <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4718,6 +4818,9 @@
       <c r="BA24" t="inlineStr"/>
       <c r="BB24" t="inlineStr"/>
       <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="inlineStr"/>
+      <c r="BF24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4777,18 +4880,18 @@
       <c r="AM25" t="inlineStr"/>
       <c r="AN25" t="inlineStr"/>
       <c r="AO25" t="inlineStr"/>
-      <c r="AP25" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AQ25" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AR25" t="inlineStr"/>
-      <c r="AS25" t="inlineStr"/>
+      <c r="AP25" t="inlineStr"/>
+      <c r="AQ25" t="inlineStr"/>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AT25" t="inlineStr"/>
       <c r="AU25" t="inlineStr"/>
       <c r="AV25" t="inlineStr"/>
@@ -4799,6 +4902,9 @@
       <c r="BA25" t="inlineStr"/>
       <c r="BB25" t="inlineStr"/>
       <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="inlineStr"/>
+      <c r="BF25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4864,22 +4970,25 @@
       <c r="AS26" t="inlineStr"/>
       <c r="AT26" t="inlineStr"/>
       <c r="AU26" t="inlineStr"/>
-      <c r="AV26" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AW26" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AX26" t="inlineStr"/>
-      <c r="AY26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AZ26" t="inlineStr"/>
       <c r="BA26" t="inlineStr"/>
       <c r="BB26" t="inlineStr"/>
       <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="inlineStr"/>
+      <c r="BF26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4953,6 +5062,9 @@
       <c r="BA27" t="inlineStr"/>
       <c r="BB27" t="inlineStr"/>
       <c r="BC27" t="inlineStr"/>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="inlineStr"/>
+      <c r="BF27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5034,6 +5146,9 @@
       <c r="BA28" t="inlineStr"/>
       <c r="BB28" t="inlineStr"/>
       <c r="BC28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="inlineStr"/>
+      <c r="BF28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5115,6 +5230,9 @@
       <c r="BA29" t="inlineStr"/>
       <c r="BB29" t="inlineStr"/>
       <c r="BC29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="inlineStr"/>
+      <c r="BF29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5196,6 +5314,9 @@
       <c r="BA30" t="inlineStr"/>
       <c r="BB30" t="inlineStr"/>
       <c r="BC30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="inlineStr"/>
+      <c r="BF30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5273,6 +5394,9 @@
       <c r="BA31" t="inlineStr"/>
       <c r="BB31" t="inlineStr"/>
       <c r="BC31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="inlineStr"/>
+      <c r="BF31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5350,6 +5474,9 @@
       <c r="BA32" t="inlineStr"/>
       <c r="BB32" t="inlineStr"/>
       <c r="BC32" t="inlineStr"/>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="inlineStr"/>
+      <c r="BF32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5431,6 +5558,9 @@
       <c r="BA33" t="inlineStr"/>
       <c r="BB33" t="inlineStr"/>
       <c r="BC33" t="inlineStr"/>
+      <c r="BD33" t="inlineStr"/>
+      <c r="BE33" t="inlineStr"/>
+      <c r="BF33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5508,6 +5638,9 @@
       <c r="BA34" t="inlineStr"/>
       <c r="BB34" t="inlineStr"/>
       <c r="BC34" t="inlineStr"/>
+      <c r="BD34" t="inlineStr"/>
+      <c r="BE34" t="inlineStr"/>
+      <c r="BF34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5526,7 +5659,11 @@
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
@@ -5589,6 +5726,9 @@
       <c r="BA35" t="inlineStr"/>
       <c r="BB35" t="inlineStr"/>
       <c r="BC35" t="inlineStr"/>
+      <c r="BD35" t="inlineStr"/>
+      <c r="BE35" t="inlineStr"/>
+      <c r="BF35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5666,6 +5806,9 @@
       <c r="BA36" t="inlineStr"/>
       <c r="BB36" t="inlineStr"/>
       <c r="BC36" t="inlineStr"/>
+      <c r="BD36" t="inlineStr"/>
+      <c r="BE36" t="inlineStr"/>
+      <c r="BF36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5743,6 +5886,9 @@
       <c r="BA37" t="inlineStr"/>
       <c r="BB37" t="inlineStr"/>
       <c r="BC37" t="inlineStr"/>
+      <c r="BD37" t="inlineStr"/>
+      <c r="BE37" t="inlineStr"/>
+      <c r="BF37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5802,20 +5948,20 @@
       <c r="AM38" t="inlineStr"/>
       <c r="AN38" t="inlineStr"/>
       <c r="AO38" t="inlineStr"/>
-      <c r="AP38" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AP38" t="inlineStr"/>
       <c r="AQ38" t="inlineStr"/>
-      <c r="AR38" t="inlineStr"/>
-      <c r="AS38" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AR38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AS38" t="inlineStr"/>
       <c r="AT38" t="inlineStr"/>
-      <c r="AU38" t="inlineStr"/>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AV38" t="inlineStr"/>
       <c r="AW38" t="inlineStr"/>
       <c r="AX38" t="inlineStr"/>
@@ -5824,6 +5970,9 @@
       <c r="BA38" t="inlineStr"/>
       <c r="BB38" t="inlineStr"/>
       <c r="BC38" t="inlineStr"/>
+      <c r="BD38" t="inlineStr"/>
+      <c r="BE38" t="inlineStr"/>
+      <c r="BF38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5884,18 +6033,18 @@
       <c r="AN39" t="inlineStr"/>
       <c r="AO39" t="inlineStr"/>
       <c r="AP39" t="inlineStr"/>
-      <c r="AQ39" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AR39" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AS39" t="inlineStr"/>
-      <c r="AT39" t="inlineStr"/>
+      <c r="AQ39" t="inlineStr"/>
+      <c r="AR39" t="inlineStr"/>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AU39" t="inlineStr"/>
       <c r="AV39" t="inlineStr"/>
       <c r="AW39" t="inlineStr"/>
@@ -5904,7 +6053,10 @@
       <c r="AZ39" t="inlineStr"/>
       <c r="BA39" t="inlineStr"/>
       <c r="BB39" t="inlineStr"/>
-      <c r="BC39" t="inlineStr">
+      <c r="BC39" t="inlineStr"/>
+      <c r="BD39" t="inlineStr"/>
+      <c r="BE39" t="inlineStr"/>
+      <c r="BF39" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -5942,7 +6094,11 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr"/>
@@ -5959,8 +6115,16 @@
       <c r="AH40" t="inlineStr"/>
       <c r="AI40" t="inlineStr"/>
       <c r="AJ40" t="inlineStr"/>
-      <c r="AK40" t="inlineStr"/>
-      <c r="AL40" t="inlineStr"/>
+      <c r="AK40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AM40" t="inlineStr"/>
       <c r="AN40" t="inlineStr"/>
       <c r="AO40" t="inlineStr"/>
@@ -5978,6 +6142,9 @@
       <c r="BA40" t="inlineStr"/>
       <c r="BB40" t="inlineStr"/>
       <c r="BC40" t="inlineStr"/>
+      <c r="BD40" t="inlineStr"/>
+      <c r="BE40" t="inlineStr"/>
+      <c r="BF40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6002,7 +6169,11 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
@@ -6021,15 +6192,27 @@
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr"/>
-      <c r="AD41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AE41" t="inlineStr"/>
       <c r="AF41" t="inlineStr"/>
       <c r="AG41" t="inlineStr"/>
-      <c r="AH41" t="inlineStr"/>
+      <c r="AH41" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AI41" t="inlineStr"/>
       <c r="AJ41" t="inlineStr"/>
       <c r="AK41" t="inlineStr"/>
-      <c r="AL41" t="inlineStr"/>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AM41" t="inlineStr"/>
       <c r="AN41" t="inlineStr"/>
       <c r="AO41" t="inlineStr"/>
@@ -6047,6 +6230,9 @@
       <c r="BA41" t="inlineStr"/>
       <c r="BB41" t="inlineStr"/>
       <c r="BC41" t="inlineStr"/>
+      <c r="BD41" t="inlineStr"/>
+      <c r="BE41" t="inlineStr"/>
+      <c r="BF41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6090,15 +6276,27 @@
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr"/>
       <c r="AC42" t="inlineStr"/>
-      <c r="AD42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AE42" t="inlineStr"/>
       <c r="AF42" t="inlineStr"/>
       <c r="AG42" t="inlineStr"/>
-      <c r="AH42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AI42" t="inlineStr"/>
       <c r="AJ42" t="inlineStr"/>
       <c r="AK42" t="inlineStr"/>
-      <c r="AL42" t="inlineStr"/>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AM42" t="inlineStr"/>
       <c r="AN42" t="inlineStr"/>
       <c r="AO42" t="inlineStr"/>
@@ -6116,6 +6314,9 @@
       <c r="BA42" t="inlineStr"/>
       <c r="BB42" t="inlineStr"/>
       <c r="BC42" t="inlineStr"/>
+      <c r="BD42" t="inlineStr"/>
+      <c r="BE42" t="inlineStr"/>
+      <c r="BF42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6141,7 +6342,11 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
@@ -6163,11 +6368,19 @@
       <c r="AE43" t="inlineStr"/>
       <c r="AF43" t="inlineStr"/>
       <c r="AG43" t="inlineStr"/>
-      <c r="AH43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AI43" t="inlineStr"/>
       <c r="AJ43" t="inlineStr"/>
       <c r="AK43" t="inlineStr"/>
-      <c r="AL43" t="inlineStr"/>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AM43" t="inlineStr"/>
       <c r="AN43" t="inlineStr"/>
       <c r="AO43" t="inlineStr"/>
@@ -6185,6 +6398,13 @@
       <c r="BA43" t="inlineStr"/>
       <c r="BB43" t="inlineStr"/>
       <c r="BC43" t="inlineStr"/>
+      <c r="BD43" t="inlineStr"/>
+      <c r="BE43" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="BF43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6245,27 +6465,30 @@
       <c r="AR44" t="inlineStr"/>
       <c r="AS44" t="inlineStr"/>
       <c r="AT44" t="inlineStr"/>
-      <c r="AU44" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AV44" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AW44" t="inlineStr"/>
-      <c r="AX44" t="inlineStr"/>
+      <c r="AU44" t="inlineStr"/>
+      <c r="AV44" t="inlineStr"/>
+      <c r="AW44" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AX44" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AY44" t="inlineStr"/>
-      <c r="AZ44" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AZ44" t="inlineStr"/>
       <c r="BA44" t="inlineStr"/>
-      <c r="BB44" t="inlineStr"/>
+      <c r="BB44" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BC44" t="inlineStr"/>
+      <c r="BD44" t="inlineStr"/>
+      <c r="BE44" t="inlineStr"/>
+      <c r="BF44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6329,24 +6552,27 @@
       <c r="AQ45" t="inlineStr"/>
       <c r="AR45" t="inlineStr"/>
       <c r="AS45" t="inlineStr"/>
-      <c r="AT45" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AU45" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AV45" t="inlineStr"/>
-      <c r="AW45" t="inlineStr"/>
+      <c r="AT45" t="inlineStr"/>
+      <c r="AU45" t="inlineStr"/>
+      <c r="AV45" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AW45" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AX45" t="inlineStr"/>
       <c r="AY45" t="inlineStr"/>
       <c r="AZ45" t="inlineStr"/>
       <c r="BA45" t="inlineStr"/>
       <c r="BB45" t="inlineStr"/>
-      <c r="BC45" t="inlineStr">
+      <c r="BC45" t="inlineStr"/>
+      <c r="BD45" t="inlineStr"/>
+      <c r="BE45" t="inlineStr"/>
+      <c r="BF45" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -6410,28 +6636,31 @@
       <c r="AQ46" t="inlineStr"/>
       <c r="AR46" t="inlineStr"/>
       <c r="AS46" t="inlineStr"/>
-      <c r="AT46" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AT46" t="inlineStr"/>
       <c r="AU46" t="inlineStr"/>
-      <c r="AV46" t="inlineStr"/>
+      <c r="AV46" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AW46" t="inlineStr"/>
       <c r="AX46" t="inlineStr"/>
-      <c r="AY46" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AZ46" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="BA46" t="inlineStr"/>
-      <c r="BB46" t="inlineStr"/>
-      <c r="BC46" t="inlineStr">
+      <c r="AY46" t="inlineStr"/>
+      <c r="AZ46" t="inlineStr"/>
+      <c r="BA46" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="BB46" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="BC46" t="inlineStr"/>
+      <c r="BD46" t="inlineStr"/>
+      <c r="BE46" t="inlineStr"/>
+      <c r="BF46" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -6469,7 +6698,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
@@ -6499,24 +6732,27 @@
       <c r="AQ47" t="inlineStr"/>
       <c r="AR47" t="inlineStr"/>
       <c r="AS47" t="inlineStr"/>
-      <c r="AT47" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AU47" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AV47" t="inlineStr"/>
-      <c r="AW47" t="inlineStr"/>
+      <c r="AT47" t="inlineStr"/>
+      <c r="AU47" t="inlineStr"/>
+      <c r="AV47" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AW47" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AX47" t="inlineStr"/>
       <c r="AY47" t="inlineStr"/>
       <c r="AZ47" t="inlineStr"/>
       <c r="BA47" t="inlineStr"/>
       <c r="BB47" t="inlineStr"/>
-      <c r="BC47" t="inlineStr">
+      <c r="BC47" t="inlineStr"/>
+      <c r="BD47" t="inlineStr"/>
+      <c r="BE47" t="inlineStr"/>
+      <c r="BF47" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -6554,7 +6790,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
@@ -6585,23 +6825,26 @@
       <c r="AR48" t="inlineStr"/>
       <c r="AS48" t="inlineStr"/>
       <c r="AT48" t="inlineStr"/>
-      <c r="AU48" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AU48" t="inlineStr"/>
       <c r="AV48" t="inlineStr"/>
-      <c r="AW48" t="inlineStr"/>
+      <c r="AW48" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AX48" t="inlineStr"/>
       <c r="AY48" t="inlineStr"/>
-      <c r="AZ48" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AZ48" t="inlineStr"/>
       <c r="BA48" t="inlineStr"/>
-      <c r="BB48" t="inlineStr"/>
-      <c r="BC48" t="inlineStr">
+      <c r="BB48" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="BC48" t="inlineStr"/>
+      <c r="BD48" t="inlineStr"/>
+      <c r="BE48" t="inlineStr"/>
+      <c r="BF48" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -6636,7 +6879,11 @@
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr"/>
@@ -6657,20 +6904,20 @@
       <c r="AI49" t="inlineStr"/>
       <c r="AJ49" t="inlineStr"/>
       <c r="AK49" t="inlineStr"/>
-      <c r="AL49" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AL49" t="inlineStr"/>
       <c r="AM49" t="inlineStr"/>
-      <c r="AN49" t="inlineStr"/>
-      <c r="AO49" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AN49" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AO49" t="inlineStr"/>
       <c r="AP49" t="inlineStr"/>
-      <c r="AQ49" t="inlineStr"/>
+      <c r="AQ49" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AR49" t="inlineStr"/>
       <c r="AS49" t="inlineStr"/>
       <c r="AT49" t="inlineStr"/>
@@ -6678,15 +6925,18 @@
       <c r="AV49" t="inlineStr"/>
       <c r="AW49" t="inlineStr"/>
       <c r="AX49" t="inlineStr"/>
-      <c r="AY49" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AY49" t="inlineStr"/>
       <c r="AZ49" t="inlineStr"/>
-      <c r="BA49" t="inlineStr"/>
+      <c r="BA49" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BB49" t="inlineStr"/>
       <c r="BC49" t="inlineStr"/>
+      <c r="BD49" t="inlineStr"/>
+      <c r="BE49" t="inlineStr"/>
+      <c r="BF49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6763,15 +7013,18 @@
       <c r="AV50" t="inlineStr"/>
       <c r="AW50" t="inlineStr"/>
       <c r="AX50" t="inlineStr"/>
-      <c r="AY50" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AY50" t="inlineStr"/>
       <c r="AZ50" t="inlineStr"/>
-      <c r="BA50" t="inlineStr"/>
+      <c r="BA50" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BB50" t="inlineStr"/>
       <c r="BC50" t="inlineStr"/>
+      <c r="BD50" t="inlineStr"/>
+      <c r="BE50" t="inlineStr"/>
+      <c r="BF50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6826,18 +7079,18 @@
       <c r="AH51" t="inlineStr"/>
       <c r="AI51" t="inlineStr"/>
       <c r="AJ51" t="inlineStr"/>
-      <c r="AK51" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AL51" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AM51" t="inlineStr"/>
-      <c r="AN51" t="inlineStr"/>
+      <c r="AK51" t="inlineStr"/>
+      <c r="AL51" t="inlineStr"/>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AN51" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AO51" t="inlineStr"/>
       <c r="AP51" t="inlineStr"/>
       <c r="AQ51" t="inlineStr"/>
@@ -6848,15 +7101,18 @@
       <c r="AV51" t="inlineStr"/>
       <c r="AW51" t="inlineStr"/>
       <c r="AX51" t="inlineStr"/>
-      <c r="AY51" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AY51" t="inlineStr"/>
       <c r="AZ51" t="inlineStr"/>
-      <c r="BA51" t="inlineStr"/>
+      <c r="BA51" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BB51" t="inlineStr"/>
       <c r="BC51" t="inlineStr"/>
+      <c r="BD51" t="inlineStr"/>
+      <c r="BE51" t="inlineStr"/>
+      <c r="BF51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6887,7 +7143,11 @@
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
@@ -6907,18 +7167,18 @@
       <c r="AH52" t="inlineStr"/>
       <c r="AI52" t="inlineStr"/>
       <c r="AJ52" t="inlineStr"/>
-      <c r="AK52" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AL52" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AM52" t="inlineStr"/>
-      <c r="AN52" t="inlineStr"/>
+      <c r="AK52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr"/>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AO52" t="inlineStr"/>
       <c r="AP52" t="inlineStr"/>
       <c r="AQ52" t="inlineStr"/>
@@ -6929,15 +7189,18 @@
       <c r="AV52" t="inlineStr"/>
       <c r="AW52" t="inlineStr"/>
       <c r="AX52" t="inlineStr"/>
-      <c r="AY52" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AY52" t="inlineStr"/>
       <c r="AZ52" t="inlineStr"/>
-      <c r="BA52" t="inlineStr"/>
+      <c r="BA52" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BB52" t="inlineStr"/>
       <c r="BC52" t="inlineStr"/>
+      <c r="BD52" t="inlineStr"/>
+      <c r="BE52" t="inlineStr"/>
+      <c r="BF52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6999,13 +7262,13 @@
       <c r="AK53" t="inlineStr"/>
       <c r="AL53" t="inlineStr"/>
       <c r="AM53" t="inlineStr"/>
-      <c r="AN53" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AN53" t="inlineStr"/>
       <c r="AO53" t="inlineStr"/>
-      <c r="AP53" t="inlineStr"/>
+      <c r="AP53" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AQ53" t="inlineStr"/>
       <c r="AR53" t="inlineStr"/>
       <c r="AS53" t="inlineStr"/>
@@ -7019,6 +7282,9 @@
       <c r="BA53" t="inlineStr"/>
       <c r="BB53" t="inlineStr"/>
       <c r="BC53" t="inlineStr"/>
+      <c r="BD53" t="inlineStr"/>
+      <c r="BE53" t="inlineStr"/>
+      <c r="BF53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7076,13 +7342,13 @@
       <c r="AK54" t="inlineStr"/>
       <c r="AL54" t="inlineStr"/>
       <c r="AM54" t="inlineStr"/>
-      <c r="AN54" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AN54" t="inlineStr"/>
       <c r="AO54" t="inlineStr"/>
-      <c r="AP54" t="inlineStr"/>
+      <c r="AP54" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AQ54" t="inlineStr"/>
       <c r="AR54" t="inlineStr"/>
       <c r="AS54" t="inlineStr"/>
@@ -7096,6 +7362,9 @@
       <c r="BA54" t="inlineStr"/>
       <c r="BB54" t="inlineStr"/>
       <c r="BC54" t="inlineStr"/>
+      <c r="BD54" t="inlineStr"/>
+      <c r="BE54" t="inlineStr"/>
+      <c r="BF54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7152,13 +7421,13 @@
       <c r="AJ55" t="inlineStr"/>
       <c r="AK55" t="inlineStr"/>
       <c r="AL55" t="inlineStr"/>
-      <c r="AM55" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AM55" t="inlineStr"/>
       <c r="AN55" t="inlineStr"/>
-      <c r="AO55" t="inlineStr"/>
+      <c r="AO55" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AP55" t="inlineStr"/>
       <c r="AQ55" t="inlineStr"/>
       <c r="AR55" t="inlineStr"/>
@@ -7173,6 +7442,9 @@
       <c r="BA55" t="inlineStr"/>
       <c r="BB55" t="inlineStr"/>
       <c r="BC55" t="inlineStr"/>
+      <c r="BD55" t="inlineStr"/>
+      <c r="BE55" t="inlineStr"/>
+      <c r="BF55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7230,13 +7502,13 @@
       <c r="AK56" t="inlineStr"/>
       <c r="AL56" t="inlineStr"/>
       <c r="AM56" t="inlineStr"/>
-      <c r="AN56" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AN56" t="inlineStr"/>
       <c r="AO56" t="inlineStr"/>
-      <c r="AP56" t="inlineStr"/>
+      <c r="AP56" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AQ56" t="inlineStr"/>
       <c r="AR56" t="inlineStr"/>
       <c r="AS56" t="inlineStr"/>
@@ -7250,6 +7522,9 @@
       <c r="BA56" t="inlineStr"/>
       <c r="BB56" t="inlineStr"/>
       <c r="BC56" t="inlineStr"/>
+      <c r="BD56" t="inlineStr"/>
+      <c r="BE56" t="inlineStr"/>
+      <c r="BF56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7327,6 +7602,9 @@
       <c r="BA57" t="inlineStr"/>
       <c r="BB57" t="inlineStr"/>
       <c r="BC57" t="inlineStr"/>
+      <c r="BD57" t="inlineStr"/>
+      <c r="BE57" t="inlineStr"/>
+      <c r="BF57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7388,13 +7666,13 @@
       <c r="AK58" t="inlineStr"/>
       <c r="AL58" t="inlineStr"/>
       <c r="AM58" t="inlineStr"/>
-      <c r="AN58" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AN58" t="inlineStr"/>
       <c r="AO58" t="inlineStr"/>
-      <c r="AP58" t="inlineStr"/>
+      <c r="AP58" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AQ58" t="inlineStr"/>
       <c r="AR58" t="inlineStr"/>
       <c r="AS58" t="inlineStr"/>
@@ -7408,6 +7686,9 @@
       <c r="BA58" t="inlineStr"/>
       <c r="BB58" t="inlineStr"/>
       <c r="BC58" t="inlineStr"/>
+      <c r="BD58" t="inlineStr"/>
+      <c r="BE58" t="inlineStr"/>
+      <c r="BF58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7465,13 +7746,13 @@
       <c r="AK59" t="inlineStr"/>
       <c r="AL59" t="inlineStr"/>
       <c r="AM59" t="inlineStr"/>
-      <c r="AN59" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AN59" t="inlineStr"/>
       <c r="AO59" t="inlineStr"/>
-      <c r="AP59" t="inlineStr"/>
+      <c r="AP59" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AQ59" t="inlineStr"/>
       <c r="AR59" t="inlineStr"/>
       <c r="AS59" t="inlineStr"/>
@@ -7485,6 +7766,9 @@
       <c r="BA59" t="inlineStr"/>
       <c r="BB59" t="inlineStr"/>
       <c r="BC59" t="inlineStr"/>
+      <c r="BD59" t="inlineStr"/>
+      <c r="BE59" t="inlineStr"/>
+      <c r="BF59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7523,7 +7807,11 @@
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
@@ -7557,15 +7845,18 @@
       <c r="AV60" t="inlineStr"/>
       <c r="AW60" t="inlineStr"/>
       <c r="AX60" t="inlineStr"/>
-      <c r="AY60" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AY60" t="inlineStr"/>
       <c r="AZ60" t="inlineStr"/>
-      <c r="BA60" t="inlineStr"/>
+      <c r="BA60" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BB60" t="inlineStr"/>
       <c r="BC60" t="inlineStr"/>
+      <c r="BD60" t="inlineStr"/>
+      <c r="BE60" t="inlineStr"/>
+      <c r="BF60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7622,13 +7913,13 @@
       <c r="AJ61" t="inlineStr"/>
       <c r="AK61" t="inlineStr"/>
       <c r="AL61" t="inlineStr"/>
-      <c r="AM61" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AM61" t="inlineStr"/>
       <c r="AN61" t="inlineStr"/>
-      <c r="AO61" t="inlineStr"/>
+      <c r="AO61" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AP61" t="inlineStr"/>
       <c r="AQ61" t="inlineStr"/>
       <c r="AR61" t="inlineStr"/>
@@ -7643,6 +7934,9 @@
       <c r="BA61" t="inlineStr"/>
       <c r="BB61" t="inlineStr"/>
       <c r="BC61" t="inlineStr"/>
+      <c r="BD61" t="inlineStr"/>
+      <c r="BE61" t="inlineStr"/>
+      <c r="BF61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7700,13 +7994,13 @@
       <c r="AK62" t="inlineStr"/>
       <c r="AL62" t="inlineStr"/>
       <c r="AM62" t="inlineStr"/>
-      <c r="AN62" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AN62" t="inlineStr"/>
       <c r="AO62" t="inlineStr"/>
-      <c r="AP62" t="inlineStr"/>
+      <c r="AP62" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AQ62" t="inlineStr"/>
       <c r="AR62" t="inlineStr"/>
       <c r="AS62" t="inlineStr"/>
@@ -7720,6 +8014,9 @@
       <c r="BA62" t="inlineStr"/>
       <c r="BB62" t="inlineStr"/>
       <c r="BC62" t="inlineStr"/>
+      <c r="BD62" t="inlineStr"/>
+      <c r="BE62" t="inlineStr"/>
+      <c r="BF62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7797,6 +8094,9 @@
       <c r="BA63" t="inlineStr"/>
       <c r="BB63" t="inlineStr"/>
       <c r="BC63" t="inlineStr"/>
+      <c r="BD63" t="inlineStr"/>
+      <c r="BE63" t="inlineStr"/>
+      <c r="BF63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7863,17 +8163,20 @@
       <c r="AT64" t="inlineStr"/>
       <c r="AU64" t="inlineStr"/>
       <c r="AV64" t="inlineStr"/>
-      <c r="AW64" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AW64" t="inlineStr"/>
       <c r="AX64" t="inlineStr"/>
-      <c r="AY64" t="inlineStr"/>
+      <c r="AY64" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AZ64" t="inlineStr"/>
       <c r="BA64" t="inlineStr"/>
       <c r="BB64" t="inlineStr"/>
       <c r="BC64" t="inlineStr"/>
+      <c r="BD64" t="inlineStr"/>
+      <c r="BE64" t="inlineStr"/>
+      <c r="BF64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7939,22 +8242,25 @@
       <c r="AS65" t="inlineStr"/>
       <c r="AT65" t="inlineStr"/>
       <c r="AU65" t="inlineStr"/>
-      <c r="AV65" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AW65" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AX65" t="inlineStr"/>
-      <c r="AY65" t="inlineStr"/>
+      <c r="AV65" t="inlineStr"/>
+      <c r="AW65" t="inlineStr"/>
+      <c r="AX65" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AY65" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AZ65" t="inlineStr"/>
       <c r="BA65" t="inlineStr"/>
       <c r="BB65" t="inlineStr"/>
       <c r="BC65" t="inlineStr"/>
+      <c r="BD65" t="inlineStr"/>
+      <c r="BE65" t="inlineStr"/>
+      <c r="BF65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8010,32 +8316,35 @@
       <c r="AM66" t="inlineStr"/>
       <c r="AN66" t="inlineStr"/>
       <c r="AO66" t="inlineStr"/>
-      <c r="AP66" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AP66" t="inlineStr"/>
       <c r="AQ66" t="inlineStr"/>
-      <c r="AR66" t="inlineStr"/>
-      <c r="AS66" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AR66" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AS66" t="inlineStr"/>
       <c r="AT66" t="inlineStr"/>
-      <c r="AU66" t="inlineStr"/>
+      <c r="AU66" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AV66" t="inlineStr"/>
       <c r="AW66" t="inlineStr"/>
-      <c r="AX66" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AX66" t="inlineStr"/>
       <c r="AY66" t="inlineStr"/>
-      <c r="AZ66" t="inlineStr"/>
+      <c r="AZ66" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="BA66" t="inlineStr"/>
       <c r="BB66" t="inlineStr"/>
       <c r="BC66" t="inlineStr"/>
+      <c r="BD66" t="inlineStr"/>
+      <c r="BE66" t="inlineStr"/>
+      <c r="BF66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8097,26 +8406,29 @@
       <c r="AO67" t="inlineStr"/>
       <c r="AP67" t="inlineStr"/>
       <c r="AQ67" t="inlineStr"/>
-      <c r="AR67" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AR67" t="inlineStr"/>
       <c r="AS67" t="inlineStr"/>
-      <c r="AT67" t="inlineStr"/>
+      <c r="AT67" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AU67" t="inlineStr"/>
-      <c r="AV67" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AV67" t="inlineStr"/>
       <c r="AW67" t="inlineStr"/>
-      <c r="AX67" t="inlineStr"/>
+      <c r="AX67" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AY67" t="inlineStr"/>
       <c r="AZ67" t="inlineStr"/>
       <c r="BA67" t="inlineStr"/>
       <c r="BB67" t="inlineStr"/>
-      <c r="BC67" t="inlineStr">
+      <c r="BC67" t="inlineStr"/>
+      <c r="BD67" t="inlineStr"/>
+      <c r="BE67" t="inlineStr"/>
+      <c r="BF67" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -8135,7 +8447,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -8176,28 +8488,31 @@
       <c r="AM68" t="inlineStr"/>
       <c r="AN68" t="inlineStr"/>
       <c r="AO68" t="inlineStr"/>
-      <c r="AP68" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AP68" t="inlineStr"/>
       <c r="AQ68" t="inlineStr"/>
-      <c r="AR68" t="inlineStr"/>
+      <c r="AR68" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AS68" t="inlineStr"/>
-      <c r="AT68" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AT68" t="inlineStr"/>
       <c r="AU68" t="inlineStr"/>
-      <c r="AV68" t="inlineStr"/>
+      <c r="AV68" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AW68" t="inlineStr"/>
       <c r="AX68" t="inlineStr"/>
       <c r="AY68" t="inlineStr"/>
       <c r="AZ68" t="inlineStr"/>
       <c r="BA68" t="inlineStr"/>
       <c r="BB68" t="inlineStr"/>
-      <c r="BC68" t="inlineStr">
+      <c r="BC68" t="inlineStr"/>
+      <c r="BD68" t="inlineStr"/>
+      <c r="BE68" t="inlineStr"/>
+      <c r="BF68" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -8216,7 +8531,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -8291,6 +8606,9 @@
       <c r="BA69" t="inlineStr"/>
       <c r="BB69" t="inlineStr"/>
       <c r="BC69" t="inlineStr"/>
+      <c r="BD69" t="inlineStr"/>
+      <c r="BE69" t="inlineStr"/>
+      <c r="BF69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8305,7 +8623,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -8384,6 +8702,9 @@
       <c r="BA70" t="inlineStr"/>
       <c r="BB70" t="inlineStr"/>
       <c r="BC70" t="inlineStr"/>
+      <c r="BD70" t="inlineStr"/>
+      <c r="BE70" t="inlineStr"/>
+      <c r="BF70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8398,7 +8719,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>absent</t>
+          <t>implemented</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -8439,20 +8760,20 @@
       <c r="AM71" t="inlineStr"/>
       <c r="AN71" t="inlineStr"/>
       <c r="AO71" t="inlineStr"/>
-      <c r="AP71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AP71" t="inlineStr"/>
       <c r="AQ71" t="inlineStr"/>
-      <c r="AR71" t="inlineStr"/>
-      <c r="AS71" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AS71" t="inlineStr"/>
       <c r="AT71" t="inlineStr"/>
-      <c r="AU71" t="inlineStr"/>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AV71" t="inlineStr"/>
       <c r="AW71" t="inlineStr"/>
       <c r="AX71" t="inlineStr"/>
@@ -8460,7 +8781,10 @@
       <c r="AZ71" t="inlineStr"/>
       <c r="BA71" t="inlineStr"/>
       <c r="BB71" t="inlineStr"/>
-      <c r="BC71" t="inlineStr">
+      <c r="BC71" t="inlineStr"/>
+      <c r="BD71" t="inlineStr"/>
+      <c r="BE71" t="inlineStr"/>
+      <c r="BF71" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -8546,6 +8870,9 @@
       <c r="BA72" t="inlineStr"/>
       <c r="BB72" t="inlineStr"/>
       <c r="BC72" t="inlineStr"/>
+      <c r="BD72" t="inlineStr"/>
+      <c r="BE72" t="inlineStr"/>
+      <c r="BF72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8623,6 +8950,9 @@
       <c r="BA73" t="inlineStr"/>
       <c r="BB73" t="inlineStr"/>
       <c r="BC73" t="inlineStr"/>
+      <c r="BD73" t="inlineStr"/>
+      <c r="BE73" t="inlineStr"/>
+      <c r="BF73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8700,6 +9030,9 @@
       <c r="BA74" t="inlineStr"/>
       <c r="BB74" t="inlineStr"/>
       <c r="BC74" t="inlineStr"/>
+      <c r="BD74" t="inlineStr"/>
+      <c r="BE74" t="inlineStr"/>
+      <c r="BF74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8762,25 +9095,28 @@
       <c r="AP75" t="inlineStr"/>
       <c r="AQ75" t="inlineStr"/>
       <c r="AR75" t="inlineStr"/>
-      <c r="AS75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AS75" t="inlineStr"/>
       <c r="AT75" t="inlineStr"/>
-      <c r="AU75" t="inlineStr"/>
-      <c r="AV75" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AU75" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AV75" t="inlineStr"/>
       <c r="AW75" t="inlineStr"/>
-      <c r="AX75" t="inlineStr"/>
+      <c r="AX75" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AY75" t="inlineStr"/>
       <c r="AZ75" t="inlineStr"/>
       <c r="BA75" t="inlineStr"/>
       <c r="BB75" t="inlineStr"/>
       <c r="BC75" t="inlineStr"/>
+      <c r="BD75" t="inlineStr"/>
+      <c r="BE75" t="inlineStr"/>
+      <c r="BF75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8858,6 +9194,9 @@
       <c r="BA76" t="inlineStr"/>
       <c r="BB76" t="inlineStr"/>
       <c r="BC76" t="inlineStr"/>
+      <c r="BD76" t="inlineStr"/>
+      <c r="BE76" t="inlineStr"/>
+      <c r="BF76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8917,20 +9256,20 @@
       <c r="AM77" t="inlineStr"/>
       <c r="AN77" t="inlineStr"/>
       <c r="AO77" t="inlineStr"/>
-      <c r="AP77" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AP77" t="inlineStr"/>
       <c r="AQ77" t="inlineStr"/>
-      <c r="AR77" t="inlineStr"/>
-      <c r="AS77" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="AR77" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AS77" t="inlineStr"/>
       <c r="AT77" t="inlineStr"/>
-      <c r="AU77" t="inlineStr"/>
+      <c r="AU77" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AV77" t="inlineStr"/>
       <c r="AW77" t="inlineStr"/>
       <c r="AX77" t="inlineStr"/>
@@ -8938,7 +9277,10 @@
       <c r="AZ77" t="inlineStr"/>
       <c r="BA77" t="inlineStr"/>
       <c r="BB77" t="inlineStr"/>
-      <c r="BC77" t="inlineStr">
+      <c r="BC77" t="inlineStr"/>
+      <c r="BD77" t="inlineStr"/>
+      <c r="BE77" t="inlineStr"/>
+      <c r="BF77" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -9004,22 +9346,25 @@
       <c r="AS78" t="inlineStr"/>
       <c r="AT78" t="inlineStr"/>
       <c r="AU78" t="inlineStr"/>
-      <c r="AV78" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AW78" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AX78" t="inlineStr"/>
-      <c r="AY78" t="inlineStr"/>
+      <c r="AV78" t="inlineStr"/>
+      <c r="AW78" t="inlineStr"/>
+      <c r="AX78" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="AY78" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="AZ78" t="inlineStr"/>
       <c r="BA78" t="inlineStr"/>
       <c r="BB78" t="inlineStr"/>
-      <c r="BC78" t="inlineStr">
+      <c r="BC78" t="inlineStr"/>
+      <c r="BD78" t="inlineStr"/>
+      <c r="BE78" t="inlineStr"/>
+      <c r="BF78" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -9036,7 +9381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9783,12 +10128,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>spc:2084</t>
+          <t>spc:2078</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Tool, test, evidence, and gate taxonomy</t>
+          <t>Documentation payload projection contract</t>
         </is>
       </c>
     </row>
@@ -9800,12 +10145,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>spc:2085</t>
+          <t>spc:2080</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Boundary-scoped test selection and status synchronization</t>
+          <t>Documentation runtime parity contract</t>
         </is>
       </c>
     </row>
@@ -9817,12 +10162,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>spc:2086</t>
+          <t>spc:2084</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Runtime DDL and schema readiness lifecycle contract</t>
+          <t>Tool, test, evidence, and gate taxonomy</t>
         </is>
       </c>
     </row>
@@ -9834,12 +10179,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>spc:2088</t>
+          <t>spc:2085</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Python/Rust runtime performance evidence contract</t>
+          <t>Boundary-scoped test selection and status synchronization</t>
         </is>
       </c>
     </row>
@@ -9851,12 +10196,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>spc:2093</t>
+          <t>spc:2086</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Fully Paritable Suite Certification Boundary</t>
+          <t>Runtime DDL and schema readiness lifecycle contract</t>
         </is>
       </c>
     </row>
@@ -9868,12 +10213,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>spc:2097</t>
+          <t>spc:2088</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Transport Event Registry Contract</t>
+          <t>Python/Rust runtime performance evidence contract</t>
         </is>
       </c>
     </row>
@@ -9885,12 +10230,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>spc:2098</t>
+          <t>spc:2093</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Derived Runtime Subevent Taxonomy</t>
+          <t>Fully Paritable Suite Certification Boundary</t>
         </is>
       </c>
     </row>
@@ -9902,12 +10247,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>spc:2099</t>
+          <t>spc:2097</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>BindingSpec Event And Subevent Projection Contract</t>
+          <t>Transport Event Registry Contract</t>
         </is>
       </c>
     </row>
@@ -9919,12 +10264,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>spc:2100</t>
+          <t>spc:2098</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Scope Schema Contract</t>
+          <t>Derived Runtime Subevent Taxonomy</t>
         </is>
       </c>
     </row>
@@ -9936,12 +10281,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>spc:2101</t>
+          <t>spc:2099</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Kernel Anchor Extension Contract</t>
+          <t>BindingSpec Event And Subevent Projection Contract</t>
         </is>
       </c>
     </row>
@@ -9953,12 +10298,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>spc:2102</t>
+          <t>spc:2100</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Protocol Phase Tree Contract</t>
+          <t>Scope Schema Contract</t>
         </is>
       </c>
     </row>
@@ -9970,12 +10315,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>spc:2103</t>
+          <t>spc:2101</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Loop Region Contract</t>
+          <t>Kernel Anchor Extension Contract</t>
         </is>
       </c>
     </row>
@@ -9987,12 +10332,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>spc:2104</t>
+          <t>spc:2102</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Yield Iterator Producer Contract</t>
+          <t>Protocol Phase Tree Contract</t>
         </is>
       </c>
     </row>
@@ -10004,12 +10349,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>spc:2109</t>
+          <t>spc:2103</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Static File Atom Chain Contract</t>
+          <t>Loop Region Contract</t>
         </is>
       </c>
     </row>
@@ -10021,12 +10366,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>spc:2114</t>
+          <t>spc:2104</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Protocol Executor Parity Evidence Contract</t>
+          <t>Yield Iterator Producer Contract</t>
         </is>
       </c>
     </row>
@@ -10038,12 +10383,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>spc:2115</t>
+          <t>spc:2109</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Typed Ok/Err Edge And ErrorCtx Contract</t>
+          <t>Static File Atom Chain Contract</t>
         </is>
       </c>
     </row>
@@ -10055,12 +10400,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>spc:2117</t>
+          <t>spc:2114</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>EventKey And Bit-Coded Dispatch Contract</t>
+          <t>Protocol Executor Parity Evidence Contract</t>
         </is>
       </c>
     </row>
@@ -10072,12 +10417,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>spc:2119</t>
+          <t>spc:2115</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Subevent Handler Contract</t>
+          <t>Typed Ok/Err Edge And ErrorCtx Contract</t>
         </is>
       </c>
     </row>
@@ -10089,10 +10434,61 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>spc:2117</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>EventKey And Bit-Coded Dispatch Contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>additional_spec</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>spc:2119</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Subevent Handler Contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>additional_spec</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>spc:2123</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Decorator Surface Contract For Eventful Protocols</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>additional_spec</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>spc:2142</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>XFail Closure Boundary And Proof Contract</t>
         </is>

</xml_diff>